<commit_message>
Add SNV headcount quarterly data
</commit_message>
<xml_diff>
--- a/图片识别季度口径数据.xlsx
+++ b/图片识别季度口径数据.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" r:id="R9b43b652807942ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly" sheetId="2" r:id="Rddf376461e8d4b8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" r:id="Rdd0f4d76f31f477a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly" sheetId="2" r:id="R441471a5e9eb434e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comp" sheetId="3" r:id="R3f18eec0c6ac486a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,11 +15,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="4">
+  <x:numFmts count="5">
     <x:numFmt numFmtId="200" formatCode="m/d/yyyy"/>
     <x:numFmt numFmtId="201" formatCode="#,##0"/>
     <x:numFmt numFmtId="202" formatCode="#,##0.##"/>
     <x:numFmt numFmtId="203" formatCode="#,##0.00"/>
+    <x:numFmt numFmtId="204" formatCode="0"/>
   </x:numFmts>
   <x:fonts count="5">
     <x:font>
@@ -49,12 +51,17 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="5">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -193,7 +200,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="45">
+  <x:cellXfs count="55">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -315,6 +322,30 @@
     <x:xf numFmtId="203" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -347,14 +378,26 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="QuarterlyDataTable" displayName="QuarterlyDataTable" ref="A5:E65" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:E65"/>
-  <x:tableColumns count="5">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="QuarterlyDataTable" displayName="QuarterlyDataTable" ref="A5:F65" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:F65"/>
+  <x:tableColumns count="6">
     <x:tableColumn id="1" name="季度"/>
     <x:tableColumn id="2" name="季度末日期"/>
     <x:tableColumn id="3" name="Asset_SNV 季度末"/>
     <x:tableColumn id="4" name="Asset_SNV 三个月平均"/>
     <x:tableColumn id="5" name="OCC_Exp_SNV 季度末"/>
+    <x:tableColumn id="6" name="SNV_HC（员工人数）"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CompDataTable" displayName="CompDataTable" ref="A1:B61" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:B61"/>
+  <x:tableColumns count="2">
+    <x:tableColumn id="1" name="YYYYQN"/>
+    <x:tableColumn id="2" name="SNV_HC"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -4190,8 +4233,8 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3062d6f4b56b40a9"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d73f1336af2475c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65357badba804f44"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16b4b2daccb64646"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4208,6 +4251,7 @@
     <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="2" ht="24" customHeight="1">
@@ -4221,7 +4265,7 @@
     </x:row>
     <x:row r="3" ht="19" customHeight="1">
       <x:c r="A3" s="27" t="str">
-        <x:v>口径：Asset_SNV 季度末取每季第 3 个月；三个月平均为季度内 3 个月的算术平均；OCC_Exp_SNV 取每季第 3 个月。</x:v>
+        <x:v>口径：Asset_SNV 季度末取每季第 3 个月；三个月平均为季度内 3 个月的算术平均；OCC_Exp_SNV 取每季第 3 个月；SNV_HC 为员工人数，取 Comp 表季度值。</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -4251,6 +4295,9 @@
       <x:c r="E5" s="33" t="str">
         <x:v>OCC_Exp_SNV 季度末</x:v>
       </x:c>
+      <x:c r="F5" s="54" t="str">
+        <x:v>SNV_HC（员工人数）</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="20" customHeight="1">
       <x:c r="A6" s="37" t="str">
@@ -4272,6 +4319,10 @@
         <x:f>'Data'!G4</x:f>
         <x:v>10144156.82</x:v>
       </x:c>
+      <x:c r="F6" s="39" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B6)*100+MONTH($B6),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>5362</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="20" customHeight="1">
       <x:c r="A7" s="41" t="str">
@@ -4293,6 +4344,10 @@
         <x:f>'Data'!G7</x:f>
         <x:v>9802970.07</x:v>
       </x:c>
+      <x:c r="F7" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B7)*100+MONTH($B7),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>5260</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="20" customHeight="1">
       <x:c r="A8" s="41" t="str">
@@ -4314,6 +4369,10 @@
         <x:f>'Data'!G10</x:f>
         <x:v>9180728.43</x:v>
       </x:c>
+      <x:c r="F8" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B8)*100+MONTH($B8),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>5146</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="20" customHeight="1">
       <x:c r="A9" s="41" t="str">
@@ -4335,6 +4394,10 @@
         <x:f>'Data'!G13</x:f>
         <x:v>8937839.96</x:v>
       </x:c>
+      <x:c r="F9" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B9)*100+MONTH($B9),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>5086</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="20" customHeight="1">
       <x:c r="A10" s="41" t="str">
@@ -4356,6 +4419,10 @@
         <x:f>'Data'!G16</x:f>
         <x:v>8841066.67</x:v>
       </x:c>
+      <x:c r="F10" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B10)*100+MONTH($B10),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>5022</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="20" customHeight="1">
       <x:c r="A11" s="41" t="str">
@@ -4377,6 +4444,10 @@
         <x:f>'Data'!G19</x:f>
         <x:v>8806412.91</x:v>
       </x:c>
+      <x:c r="F11" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B11)*100+MONTH($B11),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>5008</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="20" customHeight="1">
       <x:c r="A12" s="41" t="str">
@@ -4398,6 +4469,10 @@
         <x:f>'Data'!G22</x:f>
         <x:v>9080901.36</x:v>
       </x:c>
+      <x:c r="F12" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B12)*100+MONTH($B12),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4896</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="20" customHeight="1">
       <x:c r="A13" s="41" t="str">
@@ -4419,6 +4494,10 @@
         <x:f>'Data'!G25</x:f>
         <x:v>8970435.67</x:v>
       </x:c>
+      <x:c r="F13" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B13)*100+MONTH($B13),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4822</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="20" customHeight="1">
       <x:c r="A14" s="41" t="str">
@@ -4440,6 +4519,10 @@
         <x:f>'Data'!G28</x:f>
         <x:v>7509561.89</x:v>
       </x:c>
+      <x:c r="F14" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B14)*100+MONTH($B14),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4652</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="20" customHeight="1">
       <x:c r="A15" s="41" t="str">
@@ -4461,6 +4544,10 @@
         <x:f>'Data'!G31</x:f>
         <x:v>8553385.43</x:v>
       </x:c>
+      <x:c r="F15" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B15)*100+MONTH($B15),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4606</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="20" customHeight="1">
       <x:c r="A16" s="41" t="str">
@@ -4482,6 +4569,10 @@
         <x:f>'Data'!G34</x:f>
         <x:v>8603976.18</x:v>
       </x:c>
+      <x:c r="F16" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B16)*100+MONTH($B16),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4571</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="20" customHeight="1">
       <x:c r="A17" s="41" t="str">
@@ -4503,6 +4594,10 @@
         <x:f>'Data'!G37</x:f>
         <x:v>8685196.17</x:v>
       </x:c>
+      <x:c r="F17" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B17)*100+MONTH($B17),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4550</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="20" customHeight="1">
       <x:c r="A18" s="41" t="str">
@@ -4524,6 +4619,10 @@
         <x:f>'Data'!G40</x:f>
         <x:v>8986673.7</x:v>
       </x:c>
+      <x:c r="F18" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B18)*100+MONTH($B18),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4494</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="20" customHeight="1">
       <x:c r="A19" s="41" t="str">
@@ -4545,6 +4644,10 @@
         <x:f>'Data'!G43</x:f>
         <x:v>8934449.88</x:v>
       </x:c>
+      <x:c r="F19" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B19)*100+MONTH($B19),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4496</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="20" customHeight="1">
       <x:c r="A20" s="41" t="str">
@@ -4566,6 +4669,10 @@
         <x:f>'Data'!G46</x:f>
         <x:v>8742801.52</x:v>
       </x:c>
+      <x:c r="F20" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B20)*100+MONTH($B20),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4421</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="20" customHeight="1">
       <x:c r="A21" s="41" t="str">
@@ -4587,6 +4694,10 @@
         <x:f>'Data'!G49</x:f>
         <x:v>8242930.04</x:v>
       </x:c>
+      <x:c r="F21" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B21)*100+MONTH($B21),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4372</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="20" customHeight="1">
       <x:c r="A22" s="41" t="str">
@@ -4608,6 +4719,10 @@
         <x:f>'Data'!G52</x:f>
         <x:v>8612626.2</x:v>
       </x:c>
+      <x:c r="F22" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B22)*100+MONTH($B22),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4331</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="20" customHeight="1">
       <x:c r="A23" s="41" t="str">
@@ -4629,6 +4744,10 @@
         <x:f>'Data'!G55</x:f>
         <x:v>9183591.19</x:v>
       </x:c>
+      <x:c r="F23" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B23)*100+MONTH($B23),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4303</x:v>
+      </x:c>
     </x:row>
     <x:row r="24" ht="20" customHeight="1">
       <x:c r="A24" s="41" t="str">
@@ -4650,6 +4769,10 @@
         <x:f>'Data'!G58</x:f>
         <x:v>9065482.4</x:v>
       </x:c>
+      <x:c r="F24" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B24)*100+MONTH($B24),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4280</x:v>
+      </x:c>
     </x:row>
     <x:row r="25" ht="20" customHeight="1">
       <x:c r="A25" s="41" t="str">
@@ -4671,6 +4794,10 @@
         <x:f>'Data'!G61</x:f>
         <x:v>10345455.37</x:v>
       </x:c>
+      <x:c r="F25" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B25)*100+MONTH($B25),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4299</x:v>
+      </x:c>
     </x:row>
     <x:row r="26" ht="20" customHeight="1">
       <x:c r="A26" s="41" t="str">
@@ -4692,6 +4819,10 @@
         <x:f>'Data'!G64</x:f>
         <x:v>9430023.23</x:v>
       </x:c>
+      <x:c r="F26" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B26)*100+MONTH($B26),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4221</x:v>
+      </x:c>
     </x:row>
     <x:row r="27" ht="20" customHeight="1">
       <x:c r="A27" s="41" t="str">
@@ -4713,6 +4844,10 @@
         <x:f>'Data'!G67</x:f>
         <x:v>8842899.39</x:v>
       </x:c>
+      <x:c r="F27" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B27)*100+MONTH($B27),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4213</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="20" customHeight="1">
       <x:c r="A28" s="41" t="str">
@@ -4734,6 +4869,10 @@
         <x:f>'Data'!G70</x:f>
         <x:v>9369119.04</x:v>
       </x:c>
+      <x:c r="F28" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B28)*100+MONTH($B28),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4187</x:v>
+      </x:c>
     </x:row>
     <x:row r="29" ht="20" customHeight="1">
       <x:c r="A29" s="41" t="str">
@@ -4755,6 +4894,10 @@
         <x:f>'Data'!G73</x:f>
         <x:v>9176065.56</x:v>
       </x:c>
+      <x:c r="F29" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B29)*100+MONTH($B29),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4269</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" ht="20" customHeight="1">
       <x:c r="A30" s="41" t="str">
@@ -4776,6 +4919,10 @@
         <x:f>'Data'!G76</x:f>
         <x:v>10151828.85</x:v>
       </x:c>
+      <x:c r="F30" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B30)*100+MONTH($B30),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4284</x:v>
+      </x:c>
     </x:row>
     <x:row r="31" ht="20" customHeight="1">
       <x:c r="A31" s="41" t="str">
@@ -4797,6 +4944,10 @@
         <x:f>'Data'!G79</x:f>
         <x:v>9971043.05</x:v>
       </x:c>
+      <x:c r="F31" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B31)*100+MONTH($B31),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4272</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="20" customHeight="1">
       <x:c r="A32" s="41" t="str">
@@ -4818,6 +4969,10 @@
         <x:f>'Data'!G82</x:f>
         <x:v>9154869.21</x:v>
       </x:c>
+      <x:c r="F32" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B32)*100+MONTH($B32),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4313</x:v>
+      </x:c>
     </x:row>
     <x:row r="33" ht="20" customHeight="1">
       <x:c r="A33" s="41" t="str">
@@ -4839,6 +4994,10 @@
         <x:f>'Data'!G85</x:f>
         <x:v>9249601.21</x:v>
       </x:c>
+      <x:c r="F33" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B33)*100+MONTH($B33),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4352</x:v>
+      </x:c>
     </x:row>
     <x:row r="34" ht="20" customHeight="1">
       <x:c r="A34" s="41" t="str">
@@ -4860,6 +5019,10 @@
         <x:f>'Data'!G88</x:f>
         <x:v>10509583.11</x:v>
       </x:c>
+      <x:c r="F34" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B34)*100+MONTH($B34),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4384</x:v>
+      </x:c>
     </x:row>
     <x:row r="35" ht="20" customHeight="1">
       <x:c r="A35" s="41" t="str">
@@ -4881,6 +5044,10 @@
         <x:f>'Data'!G91</x:f>
         <x:v>10840462.06</x:v>
       </x:c>
+      <x:c r="F35" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B35)*100+MONTH($B35),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4411</x:v>
+      </x:c>
     </x:row>
     <x:row r="36" ht="20" customHeight="1">
       <x:c r="A36" s="41" t="str">
@@ -4902,6 +5069,10 @@
         <x:f>'Data'!G94</x:f>
         <x:v>10948496.88</x:v>
       </x:c>
+      <x:c r="F36" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B36)*100+MONTH($B36),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4434</x:v>
+      </x:c>
     </x:row>
     <x:row r="37" ht="20" customHeight="1">
       <x:c r="A37" s="41" t="str">
@@ -4923,6 +5094,10 @@
         <x:f>'Data'!G97</x:f>
         <x:v>11173258.78</x:v>
       </x:c>
+      <x:c r="F37" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B37)*100+MONTH($B37),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4466</x:v>
+      </x:c>
     </x:row>
     <x:row r="38" ht="20" customHeight="1">
       <x:c r="A38" s="41" t="str">
@@ -4944,6 +5119,10 @@
         <x:f>'Data'!G100</x:f>
         <x:v>13833541.18</x:v>
       </x:c>
+      <x:c r="F38" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B38)*100+MONTH($B38),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>5173</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="20" customHeight="1">
       <x:c r="A39" s="41" t="str">
@@ -4965,6 +5144,10 @@
         <x:f>'Data'!G103</x:f>
         <x:v>13251665.41</x:v>
       </x:c>
+      <x:c r="F39" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B39)*100+MONTH($B39),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>5158</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="20" customHeight="1">
       <x:c r="A40" s="41" t="str">
@@ -4986,6 +5169,10 @@
         <x:f>'Data'!G106</x:f>
         <x:v>13231966.52</x:v>
       </x:c>
+      <x:c r="F40" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B40)*100+MONTH($B40),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>5229</x:v>
+      </x:c>
     </x:row>
     <x:row r="41" ht="20" customHeight="1">
       <x:c r="A41" s="41" t="str">
@@ -5007,6 +5194,10 @@
         <x:f>'Data'!G109</x:f>
         <x:v>14620644.86</x:v>
       </x:c>
+      <x:c r="F41" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B41)*100+MONTH($B41),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>5219</x:v>
+      </x:c>
     </x:row>
     <x:row r="42" ht="20" customHeight="1">
       <x:c r="A42" s="41" t="str">
@@ -5028,6 +5219,10 @@
         <x:f>'Data'!G112</x:f>
         <x:v>14389193.29</x:v>
       </x:c>
+      <x:c r="F42" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B42)*100+MONTH($B42),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>5302</x:v>
+      </x:c>
     </x:row>
     <x:row r="43" ht="20" customHeight="1">
       <x:c r="A43" s="41" t="str">
@@ -5049,6 +5244,10 @@
         <x:f>'Data'!G115</x:f>
         <x:v>13686857.48</x:v>
       </x:c>
+      <x:c r="F43" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B43)*100+MONTH($B43),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>5308</x:v>
+      </x:c>
     </x:row>
     <x:row r="44" ht="20" customHeight="1">
       <x:c r="A44" s="41" t="str">
@@ -5070,6 +5269,10 @@
         <x:f>'Data'!G118</x:f>
         <x:v>14407656.2</x:v>
       </x:c>
+      <x:c r="F44" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B44)*100+MONTH($B44),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>5232</x:v>
+      </x:c>
     </x:row>
     <x:row r="45" ht="20" customHeight="1">
       <x:c r="A45" s="41" t="str">
@@ -5091,6 +5294,10 @@
         <x:f>'Data'!G121</x:f>
         <x:v>15273819.76</x:v>
       </x:c>
+      <x:c r="F45" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B45)*100+MONTH($B45),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>5134</x:v>
+      </x:c>
     </x:row>
     <x:row r="46" ht="20" customHeight="1">
       <x:c r="A46" s="41" t="str">
@@ -5112,6 +5319,10 @@
         <x:f>'Data'!G124</x:f>
         <x:v>13806228.59</x:v>
       </x:c>
+      <x:c r="F46" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B46)*100+MONTH($B46),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>5061</x:v>
+      </x:c>
     </x:row>
     <x:row r="47" ht="20" customHeight="1">
       <x:c r="A47" s="41" t="str">
@@ -5133,6 +5344,10 @@
         <x:f>'Data'!G127</x:f>
         <x:v>13763517.34</x:v>
       </x:c>
+      <x:c r="F47" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B47)*100+MONTH($B47),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4983</x:v>
+      </x:c>
     </x:row>
     <x:row r="48" ht="20" customHeight="1">
       <x:c r="A48" s="41" t="str">
@@ -5154,6 +5369,10 @@
         <x:f>'Data'!G130</x:f>
         <x:v>14843308.88</x:v>
       </x:c>
+      <x:c r="F48" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B48)*100+MONTH($B48),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4953</x:v>
+      </x:c>
     </x:row>
     <x:row r="49" ht="20" customHeight="1">
       <x:c r="A49" s="41" t="str">
@@ -5175,6 +5394,10 @@
         <x:f>'Data'!G133</x:f>
         <x:v>13371728.65</x:v>
       </x:c>
+      <x:c r="F49" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B49)*100+MONTH($B49),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4887</x:v>
+      </x:c>
     </x:row>
     <x:row r="50" ht="20" customHeight="1">
       <x:c r="A50" s="41" t="str">
@@ -5196,6 +5419,10 @@
         <x:f>'Data'!G136</x:f>
         <x:v>14232457.44</x:v>
       </x:c>
+      <x:c r="F50" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B50)*100+MONTH($B50),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4907</x:v>
+      </x:c>
     </x:row>
     <x:row r="51" ht="20" customHeight="1">
       <x:c r="A51" s="41" t="str">
@@ -5217,6 +5444,10 @@
         <x:f>'Data'!G139</x:f>
         <x:v>14926800.04</x:v>
       </x:c>
+      <x:c r="F51" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B51)*100+MONTH($B51),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>5005</x:v>
+      </x:c>
     </x:row>
     <x:row r="52" ht="20" customHeight="1">
       <x:c r="A52" s="41" t="str">
@@ -5238,6 +5469,10 @@
         <x:f>'Data'!G142</x:f>
         <x:v>14441065.25</x:v>
       </x:c>
+      <x:c r="F52" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B52)*100+MONTH($B52),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>5033</x:v>
+      </x:c>
     </x:row>
     <x:row r="53" ht="20" customHeight="1">
       <x:c r="A53" s="41" t="str">
@@ -5259,6 +5494,10 @@
         <x:f>'Data'!G145</x:f>
         <x:v>14734816.47</x:v>
       </x:c>
+      <x:c r="F53" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B53)*100+MONTH($B53),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>5027</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="20" customHeight="1">
       <x:c r="A54" s="41" t="str">
@@ -5280,6 +5519,10 @@
         <x:f>'Data'!G148</x:f>
         <x:v>14370979.11</x:v>
       </x:c>
+      <x:c r="F54" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B54)*100+MONTH($B54),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>5072</x:v>
+      </x:c>
     </x:row>
     <x:row r="55" ht="20" customHeight="1">
       <x:c r="A55" s="41" t="str">
@@ -5301,6 +5544,10 @@
         <x:f>'Data'!G151</x:f>
         <x:v>14911135.37</x:v>
       </x:c>
+      <x:c r="F55" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B55)*100+MONTH($B55),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>5097</x:v>
+      </x:c>
     </x:row>
     <x:row r="56" ht="20" customHeight="1">
       <x:c r="A56" s="41" t="str">
@@ -5322,6 +5569,10 @@
         <x:f>'Data'!G154</x:f>
         <x:v>15126431.92</x:v>
       </x:c>
+      <x:c r="F56" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B56)*100+MONTH($B56),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4916</x:v>
+      </x:c>
     </x:row>
     <x:row r="57" ht="20" customHeight="1">
       <x:c r="A57" s="41" t="str">
@@ -5343,6 +5594,10 @@
         <x:f>'Data'!G157</x:f>
         <x:v>16478054.96</x:v>
       </x:c>
+      <x:c r="F57" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B57)*100+MONTH($B57),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4798</x:v>
+      </x:c>
     </x:row>
     <x:row r="58" ht="20" customHeight="1">
       <x:c r="A58" s="41" t="str">
@@ -5364,6 +5619,10 @@
         <x:f>'Data'!G160</x:f>
         <x:v>16240238.4</x:v>
       </x:c>
+      <x:c r="F58" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B58)*100+MONTH($B58),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4732</x:v>
+      </x:c>
     </x:row>
     <x:row r="59" ht="20" customHeight="1">
       <x:c r="A59" s="41" t="str">
@@ -5385,6 +5644,10 @@
         <x:f>'Data'!G163</x:f>
         <x:v>15108299.56</x:v>
       </x:c>
+      <x:c r="F59" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B59)*100+MONTH($B59),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4726</x:v>
+      </x:c>
     </x:row>
     <x:row r="60" ht="20" customHeight="1">
       <x:c r="A60" s="41" t="str">
@@ -5406,6 +5669,10 @@
         <x:f>'Data'!G166</x:f>
         <x:v>15904636.45</x:v>
       </x:c>
+      <x:c r="F60" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B60)*100+MONTH($B60),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4728</x:v>
+      </x:c>
     </x:row>
     <x:row r="61" ht="20" customHeight="1">
       <x:c r="A61" s="41" t="str">
@@ -5427,6 +5694,10 @@
         <x:f>'Data'!G169</x:f>
         <x:v>16158704.52</x:v>
       </x:c>
+      <x:c r="F61" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B61)*100+MONTH($B61),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4696</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" ht="20" customHeight="1">
       <x:c r="A62" s="41" t="str">
@@ -5448,6 +5719,10 @@
         <x:f>'Data'!G172</x:f>
         <x:v>16818274.65</x:v>
       </x:c>
+      <x:c r="F62" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B62)*100+MONTH($B62),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4720</x:v>
+      </x:c>
     </x:row>
     <x:row r="63" ht="20" customHeight="1">
       <x:c r="A63" s="41" t="str">
@@ -5469,6 +5744,10 @@
         <x:f>'Data'!G175</x:f>
         <x:v>16306399.87</x:v>
       </x:c>
+      <x:c r="F63" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B63)*100+MONTH($B63),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4804</x:v>
+      </x:c>
     </x:row>
     <x:row r="64" ht="20" customHeight="1">
       <x:c r="A64" s="41" t="str">
@@ -5490,6 +5769,10 @@
         <x:f>'Data'!G178</x:f>
         <x:v>16166826.63</x:v>
       </x:c>
+      <x:c r="F64" s="20" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B64)*100+MONTH($B64),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4847</x:v>
+      </x:c>
     </x:row>
     <x:row r="65" ht="20" customHeight="1">
       <x:c r="A65" s="43" t="str">
@@ -5511,11 +5794,648 @@
         <x:f>'Data'!G181</x:f>
         <x:v>16385248.85</x:v>
       </x:c>
+      <x:c r="F65" s="23" t="n">
+        <x:f>INDEX('Comp'!$B$2:$B$61,MATCH(YEAR($B65)*100+MONTH($B65),'Comp'!$A$2:$A$61,0))</x:f>
+        <x:v>4838</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3194db33c3c4442d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R059519fa9aa24125"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FFD6B656"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="3" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="48" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="22" customHeight="1">
+      <x:c r="A1" s="48" t="str">
+        <x:v>YYYYQN</x:v>
+      </x:c>
+      <x:c r="B1" s="48" t="str">
+        <x:v>SNV_HC</x:v>
+      </x:c>
+      <x:c r="C1" s="1"/>
+      <x:c r="D1" s="50" t="str">
+        <x:v>来源：用户提供的两张截图。SNV_HC 为 SNV 员工人数。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="20" customHeight="1">
+      <x:c r="A2" s="49" t="n">
+        <x:v>201103</x:v>
+      </x:c>
+      <x:c r="B2" s="13" t="n">
+        <x:v>5362</x:v>
+      </x:c>
+      <x:c r="C2" s="1"/>
+      <x:c r="D2" s="1"/>
+    </x:row>
+    <x:row r="3" ht="20" customHeight="1">
+      <x:c r="A3" s="49" t="n">
+        <x:v>201106</x:v>
+      </x:c>
+      <x:c r="B3" s="13" t="n">
+        <x:v>5260</x:v>
+      </x:c>
+      <x:c r="C3" s="1"/>
+      <x:c r="D3" s="1"/>
+    </x:row>
+    <x:row r="4" ht="20" customHeight="1">
+      <x:c r="A4" s="49" t="n">
+        <x:v>201109</x:v>
+      </x:c>
+      <x:c r="B4" s="13" t="n">
+        <x:v>5146</x:v>
+      </x:c>
+      <x:c r="C4" s="1"/>
+      <x:c r="D4" s="1"/>
+    </x:row>
+    <x:row r="5" ht="20" customHeight="1">
+      <x:c r="A5" s="49" t="n">
+        <x:v>201112</x:v>
+      </x:c>
+      <x:c r="B5" s="13" t="n">
+        <x:v>5086</x:v>
+      </x:c>
+      <x:c r="C5" s="1"/>
+      <x:c r="D5" s="1"/>
+    </x:row>
+    <x:row r="6" ht="20" customHeight="1">
+      <x:c r="A6" s="49" t="n">
+        <x:v>201203</x:v>
+      </x:c>
+      <x:c r="B6" s="13" t="n">
+        <x:v>5022</x:v>
+      </x:c>
+      <x:c r="C6" s="1"/>
+      <x:c r="D6" s="1"/>
+    </x:row>
+    <x:row r="7" ht="20" customHeight="1">
+      <x:c r="A7" s="49" t="n">
+        <x:v>201206</x:v>
+      </x:c>
+      <x:c r="B7" s="13" t="n">
+        <x:v>5008</x:v>
+      </x:c>
+      <x:c r="C7" s="1"/>
+      <x:c r="D7" s="1"/>
+    </x:row>
+    <x:row r="8" ht="20" customHeight="1">
+      <x:c r="A8" s="49" t="n">
+        <x:v>201209</x:v>
+      </x:c>
+      <x:c r="B8" s="13" t="n">
+        <x:v>4896</x:v>
+      </x:c>
+      <x:c r="C8" s="1"/>
+      <x:c r="D8" s="1"/>
+    </x:row>
+    <x:row r="9" ht="20" customHeight="1">
+      <x:c r="A9" s="49" t="n">
+        <x:v>201212</x:v>
+      </x:c>
+      <x:c r="B9" s="13" t="n">
+        <x:v>4822</x:v>
+      </x:c>
+      <x:c r="C9" s="1"/>
+      <x:c r="D9" s="1"/>
+    </x:row>
+    <x:row r="10" ht="20" customHeight="1">
+      <x:c r="A10" s="49" t="n">
+        <x:v>201303</x:v>
+      </x:c>
+      <x:c r="B10" s="13" t="n">
+        <x:v>4652</x:v>
+      </x:c>
+      <x:c r="C10" s="1"/>
+      <x:c r="D10" s="1"/>
+    </x:row>
+    <x:row r="11" ht="20" customHeight="1">
+      <x:c r="A11" s="49" t="n">
+        <x:v>201306</x:v>
+      </x:c>
+      <x:c r="B11" s="13" t="n">
+        <x:v>4606</x:v>
+      </x:c>
+      <x:c r="C11" s="1"/>
+      <x:c r="D11" s="1"/>
+    </x:row>
+    <x:row r="12" ht="20" customHeight="1">
+      <x:c r="A12" s="49" t="n">
+        <x:v>201309</x:v>
+      </x:c>
+      <x:c r="B12" s="13" t="n">
+        <x:v>4571</x:v>
+      </x:c>
+      <x:c r="C12" s="1"/>
+      <x:c r="D12" s="1"/>
+    </x:row>
+    <x:row r="13" ht="20" customHeight="1">
+      <x:c r="A13" s="49" t="n">
+        <x:v>201312</x:v>
+      </x:c>
+      <x:c r="B13" s="13" t="n">
+        <x:v>4550</x:v>
+      </x:c>
+      <x:c r="C13" s="1"/>
+      <x:c r="D13" s="1"/>
+    </x:row>
+    <x:row r="14" ht="20" customHeight="1">
+      <x:c r="A14" s="49" t="n">
+        <x:v>201403</x:v>
+      </x:c>
+      <x:c r="B14" s="13" t="n">
+        <x:v>4494</x:v>
+      </x:c>
+      <x:c r="C14" s="1"/>
+      <x:c r="D14" s="1"/>
+    </x:row>
+    <x:row r="15" ht="20" customHeight="1">
+      <x:c r="A15" s="49" t="n">
+        <x:v>201406</x:v>
+      </x:c>
+      <x:c r="B15" s="13" t="n">
+        <x:v>4496</x:v>
+      </x:c>
+      <x:c r="C15" s="1"/>
+      <x:c r="D15" s="1"/>
+    </x:row>
+    <x:row r="16" ht="20" customHeight="1">
+      <x:c r="A16" s="49" t="n">
+        <x:v>201409</x:v>
+      </x:c>
+      <x:c r="B16" s="13" t="n">
+        <x:v>4421</x:v>
+      </x:c>
+      <x:c r="C16" s="1"/>
+      <x:c r="D16" s="1"/>
+    </x:row>
+    <x:row r="17" ht="20" customHeight="1">
+      <x:c r="A17" s="49" t="n">
+        <x:v>201412</x:v>
+      </x:c>
+      <x:c r="B17" s="13" t="n">
+        <x:v>4372</x:v>
+      </x:c>
+      <x:c r="C17" s="1"/>
+      <x:c r="D17" s="1"/>
+    </x:row>
+    <x:row r="18" ht="20" customHeight="1">
+      <x:c r="A18" s="49" t="n">
+        <x:v>201503</x:v>
+      </x:c>
+      <x:c r="B18" s="13" t="n">
+        <x:v>4331</x:v>
+      </x:c>
+      <x:c r="C18" s="1"/>
+      <x:c r="D18" s="1"/>
+    </x:row>
+    <x:row r="19" ht="20" customHeight="1">
+      <x:c r="A19" s="49" t="n">
+        <x:v>201506</x:v>
+      </x:c>
+      <x:c r="B19" s="13" t="n">
+        <x:v>4303</x:v>
+      </x:c>
+      <x:c r="C19" s="1"/>
+      <x:c r="D19" s="1"/>
+    </x:row>
+    <x:row r="20" ht="20" customHeight="1">
+      <x:c r="A20" s="49" t="n">
+        <x:v>201509</x:v>
+      </x:c>
+      <x:c r="B20" s="13" t="n">
+        <x:v>4280</x:v>
+      </x:c>
+      <x:c r="C20" s="1"/>
+      <x:c r="D20" s="1"/>
+    </x:row>
+    <x:row r="21" ht="20" customHeight="1">
+      <x:c r="A21" s="49" t="n">
+        <x:v>201512</x:v>
+      </x:c>
+      <x:c r="B21" s="13" t="n">
+        <x:v>4299</x:v>
+      </x:c>
+      <x:c r="C21" s="1"/>
+      <x:c r="D21" s="1"/>
+    </x:row>
+    <x:row r="22" ht="20" customHeight="1">
+      <x:c r="A22" s="49" t="n">
+        <x:v>201603</x:v>
+      </x:c>
+      <x:c r="B22" s="13" t="n">
+        <x:v>4221</x:v>
+      </x:c>
+      <x:c r="C22" s="1"/>
+      <x:c r="D22" s="1"/>
+    </x:row>
+    <x:row r="23" ht="20" customHeight="1">
+      <x:c r="A23" s="49" t="n">
+        <x:v>201606</x:v>
+      </x:c>
+      <x:c r="B23" s="13" t="n">
+        <x:v>4213</x:v>
+      </x:c>
+      <x:c r="C23" s="1"/>
+      <x:c r="D23" s="1"/>
+    </x:row>
+    <x:row r="24" ht="20" customHeight="1">
+      <x:c r="A24" s="49" t="n">
+        <x:v>201609</x:v>
+      </x:c>
+      <x:c r="B24" s="13" t="n">
+        <x:v>4187</x:v>
+      </x:c>
+      <x:c r="C24" s="1"/>
+      <x:c r="D24" s="1"/>
+    </x:row>
+    <x:row r="25" ht="20" customHeight="1">
+      <x:c r="A25" s="49" t="n">
+        <x:v>201612</x:v>
+      </x:c>
+      <x:c r="B25" s="13" t="n">
+        <x:v>4269</x:v>
+      </x:c>
+      <x:c r="C25" s="1"/>
+      <x:c r="D25" s="1"/>
+    </x:row>
+    <x:row r="26" ht="20" customHeight="1">
+      <x:c r="A26" s="49" t="n">
+        <x:v>201703</x:v>
+      </x:c>
+      <x:c r="B26" s="13" t="n">
+        <x:v>4284</x:v>
+      </x:c>
+      <x:c r="C26" s="1"/>
+      <x:c r="D26" s="1"/>
+    </x:row>
+    <x:row r="27" ht="20" customHeight="1">
+      <x:c r="A27" s="49" t="n">
+        <x:v>201706</x:v>
+      </x:c>
+      <x:c r="B27" s="13" t="n">
+        <x:v>4272</x:v>
+      </x:c>
+      <x:c r="C27" s="1"/>
+      <x:c r="D27" s="1"/>
+    </x:row>
+    <x:row r="28" ht="20" customHeight="1">
+      <x:c r="A28" s="49" t="n">
+        <x:v>201709</x:v>
+      </x:c>
+      <x:c r="B28" s="13" t="n">
+        <x:v>4313</x:v>
+      </x:c>
+      <x:c r="C28" s="1"/>
+      <x:c r="D28" s="1"/>
+    </x:row>
+    <x:row r="29" ht="20" customHeight="1">
+      <x:c r="A29" s="49" t="n">
+        <x:v>201712</x:v>
+      </x:c>
+      <x:c r="B29" s="13" t="n">
+        <x:v>4352</x:v>
+      </x:c>
+      <x:c r="C29" s="1"/>
+      <x:c r="D29" s="1"/>
+    </x:row>
+    <x:row r="30" ht="20" customHeight="1">
+      <x:c r="A30" s="49" t="n">
+        <x:v>201803</x:v>
+      </x:c>
+      <x:c r="B30" s="13" t="n">
+        <x:v>4384</x:v>
+      </x:c>
+      <x:c r="C30" s="1"/>
+      <x:c r="D30" s="1"/>
+    </x:row>
+    <x:row r="31" ht="20" customHeight="1">
+      <x:c r="A31" s="49" t="n">
+        <x:v>201806</x:v>
+      </x:c>
+      <x:c r="B31" s="13" t="n">
+        <x:v>4411</x:v>
+      </x:c>
+      <x:c r="C31" s="1"/>
+      <x:c r="D31" s="1"/>
+    </x:row>
+    <x:row r="32" ht="20" customHeight="1">
+      <x:c r="A32" s="49" t="n">
+        <x:v>201809</x:v>
+      </x:c>
+      <x:c r="B32" s="13" t="n">
+        <x:v>4434</x:v>
+      </x:c>
+      <x:c r="C32" s="1"/>
+      <x:c r="D32" s="1"/>
+    </x:row>
+    <x:row r="33" ht="20" customHeight="1">
+      <x:c r="A33" s="49" t="n">
+        <x:v>201812</x:v>
+      </x:c>
+      <x:c r="B33" s="13" t="n">
+        <x:v>4466</x:v>
+      </x:c>
+      <x:c r="C33" s="1"/>
+      <x:c r="D33" s="1"/>
+    </x:row>
+    <x:row r="34" ht="20" customHeight="1">
+      <x:c r="A34" s="49" t="n">
+        <x:v>201903</x:v>
+      </x:c>
+      <x:c r="B34" s="13" t="n">
+        <x:v>5173</x:v>
+      </x:c>
+      <x:c r="C34" s="1"/>
+      <x:c r="D34" s="1"/>
+    </x:row>
+    <x:row r="35" ht="20" customHeight="1">
+      <x:c r="A35" s="49" t="n">
+        <x:v>201906</x:v>
+      </x:c>
+      <x:c r="B35" s="13" t="n">
+        <x:v>5158</x:v>
+      </x:c>
+      <x:c r="C35" s="1"/>
+      <x:c r="D35" s="1"/>
+    </x:row>
+    <x:row r="36" ht="20" customHeight="1">
+      <x:c r="A36" s="49" t="n">
+        <x:v>201909</x:v>
+      </x:c>
+      <x:c r="B36" s="13" t="n">
+        <x:v>5229</x:v>
+      </x:c>
+      <x:c r="C36" s="1"/>
+      <x:c r="D36" s="1"/>
+    </x:row>
+    <x:row r="37" ht="20" customHeight="1">
+      <x:c r="A37" s="49" t="n">
+        <x:v>201912</x:v>
+      </x:c>
+      <x:c r="B37" s="13" t="n">
+        <x:v>5219</x:v>
+      </x:c>
+      <x:c r="C37" s="1"/>
+      <x:c r="D37" s="1"/>
+    </x:row>
+    <x:row r="38" ht="20" customHeight="1">
+      <x:c r="A38" s="49" t="n">
+        <x:v>202003</x:v>
+      </x:c>
+      <x:c r="B38" s="13" t="n">
+        <x:v>5302</x:v>
+      </x:c>
+      <x:c r="C38" s="1"/>
+      <x:c r="D38" s="1"/>
+    </x:row>
+    <x:row r="39" ht="20" customHeight="1">
+      <x:c r="A39" s="49" t="n">
+        <x:v>202006</x:v>
+      </x:c>
+      <x:c r="B39" s="13" t="n">
+        <x:v>5308</x:v>
+      </x:c>
+      <x:c r="C39" s="1"/>
+      <x:c r="D39" s="1"/>
+    </x:row>
+    <x:row r="40" ht="20" customHeight="1">
+      <x:c r="A40" s="49" t="n">
+        <x:v>202009</x:v>
+      </x:c>
+      <x:c r="B40" s="13" t="n">
+        <x:v>5232</x:v>
+      </x:c>
+      <x:c r="C40" s="1"/>
+      <x:c r="D40" s="1"/>
+    </x:row>
+    <x:row r="41" ht="20" customHeight="1">
+      <x:c r="A41" s="49" t="n">
+        <x:v>202012</x:v>
+      </x:c>
+      <x:c r="B41" s="13" t="n">
+        <x:v>5134</x:v>
+      </x:c>
+      <x:c r="C41" s="1"/>
+      <x:c r="D41" s="1"/>
+    </x:row>
+    <x:row r="42" ht="20" customHeight="1">
+      <x:c r="A42" s="49" t="n">
+        <x:v>202103</x:v>
+      </x:c>
+      <x:c r="B42" s="13" t="n">
+        <x:v>5061</x:v>
+      </x:c>
+      <x:c r="C42" s="1"/>
+      <x:c r="D42" s="1"/>
+    </x:row>
+    <x:row r="43" ht="20" customHeight="1">
+      <x:c r="A43" s="49" t="n">
+        <x:v>202106</x:v>
+      </x:c>
+      <x:c r="B43" s="13" t="n">
+        <x:v>4983</x:v>
+      </x:c>
+      <x:c r="C43" s="1"/>
+      <x:c r="D43" s="1"/>
+    </x:row>
+    <x:row r="44" ht="20" customHeight="1">
+      <x:c r="A44" s="49" t="n">
+        <x:v>202109</x:v>
+      </x:c>
+      <x:c r="B44" s="13" t="n">
+        <x:v>4953</x:v>
+      </x:c>
+      <x:c r="C44" s="1"/>
+      <x:c r="D44" s="1"/>
+    </x:row>
+    <x:row r="45" ht="20" customHeight="1">
+      <x:c r="A45" s="49" t="n">
+        <x:v>202112</x:v>
+      </x:c>
+      <x:c r="B45" s="13" t="n">
+        <x:v>4887</x:v>
+      </x:c>
+      <x:c r="C45" s="1"/>
+      <x:c r="D45" s="1"/>
+    </x:row>
+    <x:row r="46" ht="20" customHeight="1">
+      <x:c r="A46" s="49" t="n">
+        <x:v>202203</x:v>
+      </x:c>
+      <x:c r="B46" s="13" t="n">
+        <x:v>4907</x:v>
+      </x:c>
+      <x:c r="C46" s="1"/>
+      <x:c r="D46" s="1"/>
+    </x:row>
+    <x:row r="47" ht="20" customHeight="1">
+      <x:c r="A47" s="49" t="n">
+        <x:v>202206</x:v>
+      </x:c>
+      <x:c r="B47" s="13" t="n">
+        <x:v>5005</x:v>
+      </x:c>
+      <x:c r="C47" s="1"/>
+      <x:c r="D47" s="1"/>
+    </x:row>
+    <x:row r="48" ht="20" customHeight="1">
+      <x:c r="A48" s="49" t="n">
+        <x:v>202209</x:v>
+      </x:c>
+      <x:c r="B48" s="13" t="n">
+        <x:v>5033</x:v>
+      </x:c>
+      <x:c r="C48" s="1"/>
+      <x:c r="D48" s="1"/>
+    </x:row>
+    <x:row r="49" ht="20" customHeight="1">
+      <x:c r="A49" s="49" t="n">
+        <x:v>202212</x:v>
+      </x:c>
+      <x:c r="B49" s="13" t="n">
+        <x:v>5027</x:v>
+      </x:c>
+      <x:c r="C49" s="1"/>
+      <x:c r="D49" s="1"/>
+    </x:row>
+    <x:row r="50" ht="20" customHeight="1">
+      <x:c r="A50" s="49" t="n">
+        <x:v>202303</x:v>
+      </x:c>
+      <x:c r="B50" s="13" t="n">
+        <x:v>5072</x:v>
+      </x:c>
+      <x:c r="C50" s="1"/>
+      <x:c r="D50" s="1"/>
+    </x:row>
+    <x:row r="51" ht="20" customHeight="1">
+      <x:c r="A51" s="49" t="n">
+        <x:v>202306</x:v>
+      </x:c>
+      <x:c r="B51" s="13" t="n">
+        <x:v>5097</x:v>
+      </x:c>
+      <x:c r="C51" s="1"/>
+      <x:c r="D51" s="1"/>
+    </x:row>
+    <x:row r="52" ht="20" customHeight="1">
+      <x:c r="A52" s="49" t="n">
+        <x:v>202309</x:v>
+      </x:c>
+      <x:c r="B52" s="13" t="n">
+        <x:v>4916</x:v>
+      </x:c>
+      <x:c r="C52" s="1"/>
+      <x:c r="D52" s="1"/>
+    </x:row>
+    <x:row r="53" ht="20" customHeight="1">
+      <x:c r="A53" s="49" t="n">
+        <x:v>202312</x:v>
+      </x:c>
+      <x:c r="B53" s="13" t="n">
+        <x:v>4798</x:v>
+      </x:c>
+      <x:c r="C53" s="1"/>
+      <x:c r="D53" s="1"/>
+    </x:row>
+    <x:row r="54" ht="20" customHeight="1">
+      <x:c r="A54" s="49" t="n">
+        <x:v>202403</x:v>
+      </x:c>
+      <x:c r="B54" s="13" t="n">
+        <x:v>4732</x:v>
+      </x:c>
+      <x:c r="C54" s="1"/>
+      <x:c r="D54" s="1"/>
+    </x:row>
+    <x:row r="55" ht="20" customHeight="1">
+      <x:c r="A55" s="49" t="n">
+        <x:v>202406</x:v>
+      </x:c>
+      <x:c r="B55" s="13" t="n">
+        <x:v>4726</x:v>
+      </x:c>
+      <x:c r="C55" s="1"/>
+      <x:c r="D55" s="1"/>
+    </x:row>
+    <x:row r="56" ht="20" customHeight="1">
+      <x:c r="A56" s="49" t="n">
+        <x:v>202409</x:v>
+      </x:c>
+      <x:c r="B56" s="13" t="n">
+        <x:v>4728</x:v>
+      </x:c>
+      <x:c r="C56" s="1"/>
+      <x:c r="D56" s="1"/>
+    </x:row>
+    <x:row r="57" ht="20" customHeight="1">
+      <x:c r="A57" s="49" t="n">
+        <x:v>202412</x:v>
+      </x:c>
+      <x:c r="B57" s="13" t="n">
+        <x:v>4696</x:v>
+      </x:c>
+      <x:c r="C57" s="1"/>
+      <x:c r="D57" s="1"/>
+    </x:row>
+    <x:row r="58" ht="20" customHeight="1">
+      <x:c r="A58" s="49" t="n">
+        <x:v>202503</x:v>
+      </x:c>
+      <x:c r="B58" s="13" t="n">
+        <x:v>4720</x:v>
+      </x:c>
+      <x:c r="C58" s="1"/>
+      <x:c r="D58" s="1"/>
+    </x:row>
+    <x:row r="59" ht="20" customHeight="1">
+      <x:c r="A59" s="49" t="n">
+        <x:v>202506</x:v>
+      </x:c>
+      <x:c r="B59" s="13" t="n">
+        <x:v>4804</x:v>
+      </x:c>
+      <x:c r="C59" s="1"/>
+      <x:c r="D59" s="1"/>
+    </x:row>
+    <x:row r="60" ht="20" customHeight="1">
+      <x:c r="A60" s="49" t="n">
+        <x:v>202509</x:v>
+      </x:c>
+      <x:c r="B60" s="13" t="n">
+        <x:v>4847</x:v>
+      </x:c>
+      <x:c r="C60" s="1"/>
+      <x:c r="D60" s="1"/>
+    </x:row>
+    <x:row r="61" ht="20" customHeight="1">
+      <x:c r="A61" s="49" t="n">
+        <x:v>202512</x:v>
+      </x:c>
+      <x:c r="B61" s="13" t="n">
+        <x:v>4838</x:v>
+      </x:c>
+      <x:c r="C61" s="1"/>
+      <x:c r="D61" s="1"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra864c2f8bccc4f1c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>